<commit_message>
Updating and reorganizing Pinellas County data.
</commit_message>
<xml_diff>
--- a/Anole Dissections COPY.xlsx
+++ b/Anole Dissections COPY.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasminekesselring/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasminekesselring/Biometry-Fall-2026/Anole_Biometry_Practice/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0CAAA7-976C-3042-9AC7-F22F03EA9937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{FCE7CA0B-63A0-0549-AE67-66A5F1BD3665}"/>
+    <workbookView xWindow="3020" yWindow="660" windowWidth="29400" windowHeight="17260" activeTab="6" xr2:uid="{FCE7CA0B-63A0-0549-AE67-66A5F1BD3665}"/>
   </bookViews>
   <sheets>
     <sheet name="Everglades (Markham Park)" sheetId="12" r:id="rId1"/>

</xml_diff>